<commit_message>
Update reqs for phase 2
</commit_message>
<xml_diff>
--- a/Documents/Requirements/Requirement_Specification.xlsx
+++ b/Documents/Requirements/Requirement_Specification.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/crispin/Projects/Personal/School/Autonomous_Parking_Test/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ed6fcd04221c3a95/Desktop/Halmstad_2026/Programme/Materials/Semester_1/Network_Testing_For_Embedded_Systems_DT8076/Software_Testing/Project/JUnit/Documents/Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F38D7A02-FC59-EE45-928B-E8806CF47183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="142" documentId="13_ncr:1_{F38D7A02-FC59-EE45-928B-E8806CF47183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1B82843-E95B-4C24-B782-C5DC1085907A}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3B894777-90B3-446D-AADB-3993D3671D93}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
     <sheet name="Requirements" sheetId="2" r:id="rId2"/>
     <sheet name="Stuff" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Requirements!$A$1:$G$48</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="129">
   <si>
     <r>
       <t xml:space="preserve">Moves along a </t>
@@ -207,21 +210,12 @@
     <t>Where Is</t>
   </si>
   <si>
-    <t>R11</t>
-  </si>
-  <si>
     <t>Actuators</t>
   </si>
   <si>
     <t>Not Modeled</t>
   </si>
   <si>
-    <t>R12</t>
-  </si>
-  <si>
-    <t>Sensors</t>
-  </si>
-  <si>
     <t>R1.1</t>
   </si>
   <si>
@@ -330,9 +324,6 @@
     <t>Query the sensors using isEmpty()</t>
   </si>
   <si>
-    <t xml:space="preserve"> Move 1 m foward per step</t>
-  </si>
-  <si>
     <t>R8.1</t>
   </si>
   <si>
@@ -421,13 +412,112 @@
   </si>
   <si>
     <t>Filter value deviation &gt; 80 cm, sensor data is invalid</t>
+  </si>
+  <si>
+    <t>Read a current position before incrementing position</t>
+  </si>
+  <si>
+    <t>Move 1 m foward per step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">if sensor data returns valid, increasing one  Free Spot Length </t>
+  </si>
+  <si>
+    <t xml:space="preserve">if sensor data returns invalid, reset Free Spot Length </t>
+  </si>
+  <si>
+    <t>if sensor data returns invalid
+Free Spot Length &gt;= 5
+Current MostEfficientFreeSpot = null
+Then update MostEfficientFreeSpot</t>
+  </si>
+  <si>
+    <t>if sensor data returns invalid
+Free Spot Length &gt;= 5
+Current MostEfficientFreeSpot length &gt;  Free Spot Length
+Then update MostEfficientFreeSpot</t>
+  </si>
+  <si>
+    <t>if car position = 500
+Free Spot Length &gt;= 5
+Current MostEfficientFreeSpot length &gt;  Free Spot Length
+Then update MostEfficientFreeSpot</t>
+  </si>
+  <si>
+    <t>if car position = 500
+Free Spot Length &gt;= 5
+Current MostEfficientFreeSpot length = 0
+Then update MostEfficientFreeSpot</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>R6.5</t>
+  </si>
+  <si>
+    <t>R6.6</t>
+  </si>
+  <si>
+    <t>R6.7</t>
+  </si>
+  <si>
+    <t>R6.8</t>
+  </si>
+  <si>
+    <t>R6.9</t>
+  </si>
+  <si>
+    <t>R6.10</t>
+  </si>
+  <si>
+    <t>R6.11</t>
+  </si>
+  <si>
+    <t>Keep moving forward until car position = 500</t>
+  </si>
+  <si>
+    <t>If none of the MostEfficientFreeSpot is found, return FALSE and update status to UNPARKED</t>
+  </si>
+  <si>
+    <t>Otherwise keep moving backward until the position of the MostEfficientFreeSpot is found -&gt; update status to PARKED , RESET freeSpotsLength, MostEfficientFreeSpot, and return TRUE</t>
+  </si>
+  <si>
+    <t>R8.4</t>
+  </si>
+  <si>
+    <t>R8.5</t>
+  </si>
+  <si>
+    <t>R8.6</t>
+  </si>
+  <si>
+    <t>Increment a car position by 1</t>
+  </si>
+  <si>
+    <t>Decrement a car position by 1</t>
+  </si>
+  <si>
+    <t>Return the current car position on road</t>
+  </si>
+  <si>
+    <t>R11.2</t>
+  </si>
+  <si>
+    <t>R11.1</t>
+  </si>
+  <si>
+    <t>R11.3</t>
+  </si>
+  <si>
+    <t>R11.4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -447,6 +537,12 @@
       <strike/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -542,7 +638,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -550,12 +646,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -592,17 +682,82 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -628,10 +783,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -952,12 +1103,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BFD0E3D-BB49-40A2-B972-E4AF16E0E27F}">
   <dimension ref="A2:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="52.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -965,7 +1116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -973,7 +1124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -981,7 +1132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -989,7 +1140,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -997,7 +1148,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1005,15 +1156,15 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="14">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1028,19 +1179,20 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A83168E-7A47-49AC-91ED-2ADE1EA7B12C}">
-  <dimension ref="A1:F36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:G48"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.33203125" style="7" customWidth="1"/>
     <col min="2" max="2" width="31" style="4" customWidth="1"/>
-    <col min="3" max="3" width="17.5" customWidth="1"/>
-    <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.83203125" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
+    <col min="4" max="4" width="36.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.77734375" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6" style="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="3" t="s">
@@ -1052,68 +1204,80 @@
       <c r="D1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="8" t="s">
+      <c r="F1" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="16"/>
+      <c r="F2" s="20">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="14"/>
       <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B4" s="17"/>
+        <v>90</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" s="20">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" s="15"/>
       <c r="C4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="F4" s="20">
+        <v>1</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="16" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -1122,32 +1286,38 @@
       <c r="D5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="19"/>
+      <c r="E5" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="20">
+        <v>1</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="18"/>
       <c r="C6" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B7" s="15" t="s">
+      <c r="E6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="20">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -1156,64 +1326,76 @@
       <c r="D7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="16"/>
+      <c r="E7" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" s="20">
+        <v>1</v>
+      </c>
+      <c r="G7" s="1"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="14"/>
       <c r="C8" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="16"/>
+      <c r="E8" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F8" s="20">
+        <v>1</v>
+      </c>
+      <c r="G8" s="1"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="14"/>
       <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A10" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" s="17"/>
+      <c r="E9" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F9" s="20">
+        <v>1</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="15"/>
       <c r="C10" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="18" t="s">
+      <c r="E10" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="20">
+        <v>1</v>
+      </c>
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="16" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -1222,96 +1404,114 @@
       <c r="D11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B12" s="20"/>
+      <c r="E11" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F11" s="20">
+        <v>1</v>
+      </c>
+      <c r="G11" s="1"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="17"/>
       <c r="C12" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="20"/>
+      <c r="E12" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" s="20">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B13" s="17"/>
       <c r="C13" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="20"/>
+      <c r="E13" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="F13" s="20">
+        <v>1</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="17"/>
       <c r="C14" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B15" s="20"/>
+      <c r="E14" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="20">
+        <v>1</v>
+      </c>
+      <c r="G14" s="1"/>
+    </row>
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="17"/>
       <c r="C15" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="B16" s="19"/>
+      <c r="E15" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="F15" s="20">
+        <v>1</v>
+      </c>
+      <c r="G15" s="1"/>
+    </row>
+    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="18"/>
       <c r="C16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="15" t="s">
+      <c r="E16" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="F16" s="20">
+        <v>1</v>
+      </c>
+      <c r="G16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -1320,48 +1520,57 @@
       <c r="D17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" s="16"/>
+      <c r="E17" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" s="20">
+        <v>1</v>
+      </c>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" s="14"/>
       <c r="C18" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E18" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="17"/>
+      <c r="E18" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F18" s="20">
+        <v>1</v>
+      </c>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" s="15"/>
       <c r="C19" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="18" t="s">
+      <c r="E19" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="20">
+        <v>1</v>
+      </c>
+      <c r="G19" s="1"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="16" t="s">
         <v>22</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1370,294 +1579,583 @@
       <c r="D20" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E20" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="20"/>
+      <c r="E20" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="F20" s="20">
+        <v>1</v>
+      </c>
+      <c r="G20" s="1"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="17"/>
       <c r="C21" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E21" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A22" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B22" s="20"/>
+      <c r="E21" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F21" s="20">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1"/>
+    </row>
+    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="17"/>
       <c r="C22" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E22" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B23" s="19"/>
+      <c r="E22" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F22" s="20">
+        <v>1</v>
+      </c>
+      <c r="G22" s="1"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="17"/>
       <c r="C23" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E23" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="15" t="s">
-        <v>24</v>
-      </c>
+      <c r="E23" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F23" s="20">
+        <v>1</v>
+      </c>
+      <c r="G23" s="1"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B24" s="17"/>
       <c r="C24" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E24" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="F24" s="1"/>
-    </row>
-    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="B25" s="16"/>
+        <v>23</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="F24" s="20">
+        <v>2</v>
+      </c>
+      <c r="G24" s="1"/>
+    </row>
+    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="B25" s="17"/>
       <c r="C25" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A26" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="16"/>
+        <v>23</v>
+      </c>
+      <c r="E25" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" s="20">
+        <v>2</v>
+      </c>
+      <c r="G25" s="1"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="17"/>
       <c r="C26" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="F26" s="1"/>
-    </row>
-    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="8" t="s">
-        <v>69</v>
+        <v>23</v>
+      </c>
+      <c r="E26" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" s="20">
+        <v>2</v>
+      </c>
+      <c r="G26" s="1"/>
+    </row>
+    <row r="27" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>112</v>
       </c>
       <c r="B27" s="17"/>
       <c r="C27" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D27" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E27" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="20">
+        <v>2</v>
+      </c>
+      <c r="G27" s="1"/>
+    </row>
+    <row r="28" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B28" s="17"/>
+      <c r="C28" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E28" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F28" s="20">
+        <v>2</v>
+      </c>
+      <c r="G28" s="1"/>
+    </row>
+    <row r="29" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B29" s="17"/>
+      <c r="C29" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29" s="20">
+        <v>2</v>
+      </c>
+      <c r="G29" s="1"/>
+    </row>
+    <row r="30" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" s="18"/>
+      <c r="C30" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="F30" s="20">
+        <v>2</v>
+      </c>
+      <c r="G30" s="1"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D31" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E31" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F31" s="20">
+        <v>1</v>
+      </c>
+      <c r="G31" s="1"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="14"/>
+      <c r="C32" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="F32" s="20">
+        <v>1</v>
+      </c>
+      <c r="G32" s="1"/>
+    </row>
+    <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="8" t="s">
+      <c r="B33" s="14"/>
+      <c r="C33" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="F33" s="20">
+        <v>1</v>
+      </c>
+      <c r="G33" s="1"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" s="15"/>
+      <c r="C34" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F34" s="20">
+        <v>1</v>
+      </c>
+      <c r="G34" s="1"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F35" s="20">
+        <v>1</v>
+      </c>
+      <c r="G35" s="1"/>
+    </row>
+    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B36" s="17"/>
+      <c r="C36" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F36" s="20">
+        <v>1</v>
+      </c>
+      <c r="G36" s="1"/>
+    </row>
+    <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="B37" s="17"/>
+      <c r="C37" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="F37" s="20">
+        <v>1</v>
+      </c>
+      <c r="G37" s="1"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B38" s="17"/>
+      <c r="C38" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F38" s="20">
+        <v>2</v>
+      </c>
+      <c r="G38" s="1"/>
+    </row>
+    <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B39" s="17"/>
+      <c r="C39" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F39" s="20">
+        <v>2</v>
+      </c>
+      <c r="G39" s="1"/>
+    </row>
+    <row r="40" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B40" s="18"/>
+      <c r="C40" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="F40" s="20">
+        <v>2</v>
+      </c>
+      <c r="G40" s="1"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F41" s="20">
+        <v>1</v>
+      </c>
+      <c r="G41" s="1"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B42" s="15"/>
+      <c r="C42" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E42" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E28" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A29" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E29" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6" ht="32" x14ac:dyDescent="0.2">
-      <c r="A30" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="8" t="s">
+      <c r="F42" s="20">
+        <v>1</v>
+      </c>
+      <c r="G42" s="1"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="F43" s="20">
+        <v>1</v>
+      </c>
+      <c r="G43" s="1"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" s="18"/>
+      <c r="C44" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="8" t="s">
+      <c r="F44" s="20">
+        <v>1</v>
+      </c>
+      <c r="G44" s="1"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D45" s="1"/>
+      <c r="E45" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45" s="20">
+        <v>1</v>
+      </c>
+      <c r="G45" s="1"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B46" s="14"/>
+      <c r="C46" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="F46" s="20">
+        <v>2</v>
+      </c>
+      <c r="G46" s="1"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="B47" s="14"/>
+      <c r="C47" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="F47" s="20">
+        <v>2</v>
+      </c>
+      <c r="G47" s="1"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="B48" s="15"/>
+      <c r="C48" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B33" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E33" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="F33" s="1"/>
-    </row>
-    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B34" s="19"/>
-      <c r="C34" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="F34" s="1"/>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D35" s="1"/>
-      <c r="E35" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F35" s="1"/>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D36" s="1"/>
-      <c r="E36" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="F36" s="1"/>
+      <c r="E48" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F48" s="20">
+        <v>2</v>
+      </c>
+      <c r="G48" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="B33:B34"/>
+  <mergeCells count="11">
+    <mergeCell ref="B35:B40"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="B43:B44"/>
     <mergeCell ref="B2:B4"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="B11:B16"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B30"/>
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="B41:B42"/>
   </mergeCells>
-  <conditionalFormatting sqref="C2:C36">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Non-functional">
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="C2:C48">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="Non-functional">
       <formula>NOT(ISERROR(SEARCH("Non-functional",C2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Functional">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Functional">
       <formula>NOT(ISERROR(SEARCH("Functional",C2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F1:F1048576">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="1">
+      <formula>NOT(ISERROR(SEARCH("1",F1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="2">
+      <formula>NOT(ISERROR(SEARCH("2",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1668,7 +2166,7 @@
           <x14:formula1>
             <xm:f>Stuff!$A$1:$A$3</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C36</xm:sqref>
+          <xm:sqref>C2:C48</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1679,22 +2177,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6679FE4-DA14-4326-B96B-ACDA17B52EED}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>17</v>
       </c>

</xml_diff>